<commit_message>
English: resolve three pilot blockers in the doubling journey
A. A recognised slip no longer uses up the diagnostic budget, and the budget alone
   never leads to teaching without a rule error; running out is insufficient evidence.
B. Every reassessment after teaching includes an unfamiliar contrast (six new
   provisional items); a learner who doubles everything cannot pass.
C. The final hint is a labelled worked example recorded as revealing the answer;
   the next word is new and tried without a hint first.
Learners G and H, workbook, readiness report and demo updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015GA5TWo6ZSg3Kedq5zJW5b
</commit_message>
<xml_diff>
--- a/docs/english/review/doubling-educator-review.xlsx
+++ b/docs/english/review/doubling-educator-review.xlsx
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="497">
   <si>
     <t xml:space="preserve">OpenPath: educator review of the consonant-doubling journey</t>
   </si>
@@ -295,7 +295,7 @@
     <t xml:space="preserve">Contrast (must not double)</t>
   </si>
   <si>
-    <t xml:space="preserve">Diagnostic check only (contrast questions are not used after teaching)</t>
+    <t xml:space="preserve">Diagnostic check, or the 'must not double' word in the reassessment after each lesson (unseen only)</t>
   </si>
   <si>
     <t xml:space="preserve">Contrast: two final consonants (mp), so no doubling.</t>
@@ -424,7 +424,103 @@
     <t xml:space="preserve">Contrast: vowel team (ai), so no doubling. Correction format.</t>
   </si>
   <si>
-    <t xml:space="preserve">As 21: format may confuse. The only contrast with a vowel team.</t>
+    <t xml:space="preserve">As 21: format may confuse.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spl.infl.26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Write the past tense of melt: The ice cream ___ in the sun.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">melted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">meltted → over doubling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEW contrast for the check after teaching: two final consonants (lt).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None expected. 'melted' is a less common past tense for younger pupils.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spl.infl.27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Write the past tense of cook: Yesterday we ___ rice for dinner.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cooked</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cookked → over doubling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEW contrast: vowel team (oo).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spl.infl.28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add -est to fast: The cheetah is the ___ animal on land.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fastest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fasttest → over doubling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEW contrast: two final consonants (st); -est ending.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spl.infl.29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Write the past tense of shout: The children ___ for joy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shouted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shoutted → over doubling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEW contrast: vowel team (ou).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spl.infl.30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Write the -ing form of dream: The cat is ___ by the fire.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dreaming</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dreamming → over doubling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEW contrast: vowel team (ea).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'ea' has a short sound in some words (head, bread); here it is long. A child taught 'listen for the short vowel' may hesitate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spl.infl.31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add -er to dark: The sky grew ___ as the storm came closer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">darker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">darkker → over doubling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEW contrast: two final consonants (rk); -er ending.</t>
   </si>
   <si>
     <t xml:space="preserve">Strategy ID</t>
@@ -488,7 +584,7 @@
     <t xml:space="preserve">Learner may apply the rule to any word ending vowel + consonant, including fix → 'fixxing', snow → 'snowwing', visit → 'visitted', open → 'openning', and to consonant suffixes (sad → 'saddly').</t>
   </si>
   <si>
-    <t xml:space="preserve">The app's check: 2 unseen 'must double' questions on the learner's own, no hints. No contrast question is asked after teaching, so a learner who now doubles everything would still pass.</t>
+    <t xml:space="preserve">The app's check: 3 unseen questions on the learner's own, no hints: a word that must double, a word that must NOT double, then another that must double. All must be right for the lesson to count as having worked, so a learner who now doubles everything does not pass.</t>
   </si>
   <si>
     <t xml:space="preserve">sound_first</t>
@@ -583,16 +679,16 @@
     <t xml:space="preserve">skip ends in one vowel and one consonant (p). What happens to the p?</t>
   </si>
   <si>
-    <t xml:space="preserve">Double it: {base} + {last} + {ending}.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Double it: clap + p + ing.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Double it: skip + p + ed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gives the answer: the child only has to join three parts. Is level 3 meant to be a model answer?</t>
+    <t xml:space="preserve">Worked example (this shows the answer): {base} ends in one vowel and one consonant, so the {last} doubles: {base} + {last} + {ending} = {word}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Worked example: this shows the answer.] clap ends in one vowel and one consonant, so the p doubles: clap + p + ing = clapping.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Worked example: this shows the answer.] skip ends in one vowel and one consonant, so the p doubles: skip + p + ed = skipped.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REVISED: now a labelled worked example that shows the answer. The app records that the answer was shown; the answer typed after it is help, never independent, and the next word is new and tried once without a hint. Please check the wording.</t>
   </si>
   <si>
     <t xml:space="preserve">Say {base} out loud. Is the vowel short, as in cat or sit?</t>
@@ -616,16 +712,16 @@
     <t xml:space="preserve">States as a fact that a short vowel 'needs a guard'. True for these one-syllable words; overgeneralises beyond them.</t>
   </si>
   <si>
-    <t xml:space="preserve">{base} + {last} + {ending}.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">clap + p + ing.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">skip + p + ed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gives the answer.</t>
+    <t xml:space="preserve">Worked example (this shows the answer): say {base}, then double the {last} and add the ending: {base} + {last} + {ending} = {word}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Worked example: this shows the answer.] say clap, then double the p and add the ending: clap + p + ing = clapping.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Worked example: this shows the answer.] say skip, then double the p and add the ending: skip + p + ed = skipped.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REVISED: now a labelled worked example that shows the answer. The app records that the answer was shown; the answer typed after it is help, never independent, and the next word is new and tried once without a hint. Please check the wording. This one no longer mentions the short vowel.</t>
   </si>
   <si>
     <t xml:space="preserve">Split it: {base} | ? | {ending}. Does {base} end in one vowel and one consonant?</t>
@@ -643,6 +739,15 @@
     <t xml:space="preserve">Yes, so the middle part is another p.</t>
   </si>
   <si>
+    <t xml:space="preserve">Worked example (this shows the answer): {base} | {last} | {ending} = {word}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Worked example: this shows the answer.] clap | p | ing = clapping.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Worked example: this shows the answer.] skip | p | ed = skipped.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Root</t>
   </si>
   <si>
@@ -1096,6 +1201,45 @@
     <t xml:space="preserve">Not yet. A hint might help.</t>
   </si>
   <si>
+    <t xml:space="preserve">Not yet. A worked example can show you how.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEW: before the third hint.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hint button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Show a worked example</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEW: the third hint button.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Worked example label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Worked example: this shows the answer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEW.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Right, after seeing the worked example. Next, a new word.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A new word: try it yourself first.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEW: the word after a worked example; no hint until one try.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doubled a letter where it should not be doubled: teaching when to double, and when not to.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEW: for a learner whose only errors are doubling where it should not.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Summary</t>
   </si>
   <si>
@@ -1159,9 +1303,6 @@
     <t xml:space="preserve">Right with help in practice, not yet without help.</t>
   </si>
   <si>
-    <t xml:space="preserve">Right on new words without help after teaching. Progress, not yet mastery: more answers and a check after a week are needed.</t>
-  </si>
-  <si>
     <t xml:space="preserve">First shown on {date}; not remembered at the check after a week. Needs refreshing.</t>
   </si>
   <si>
@@ -1204,13 +1345,52 @@
     <t xml:space="preserve">{n} lesson(s) ({names}). Practice with help: {a} right at the first try, {b} right after a hint or second try, {h} hints used.</t>
   </si>
   <si>
+    <t xml:space="preserve">, of which {w} were worked examples showing the answer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEW: appended when a worked example was shown.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">right only after a worked example showed the answer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEW: end of a 'with help' line.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">not right, even after a worked example showed the answer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doubles correctly where it is needed, but also doubles where it should not. Not yet shown without help.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEW: over-doubling.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Right on new words without help after teaching, including a word that must not double. Progress, not yet mastery: more answers and a check after a week are needed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REVISED: now says a 'must not double' word was included.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Question gap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The check after the last lesson could not be finished: no unused {'must not double'} question is left. This is a gap in the app's questions, not a result about the learner; more reviewed questions are needed.</t>
+  </si>
+  <si>
     <t xml:space="preserve">None: every answer so far was given without help.</t>
   </si>
   <si>
     <t xml:space="preserve">After teaching</t>
   </si>
   <si>
-    <t xml:space="preserve">After "{strategy}": {right} of {total} new words right without help.</t>
+    <t xml:space="preserve">After "{strategy}": {right} of {total} new words right without help, and {c} of {ct} words that must not double.{ Check not finished.}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REVISED: now includes the 'must not double' word.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">After "{strategy}": not checked yet.</t>
   </si>
   <si>
     <t xml:space="preserve">Remembered later</t>
@@ -1336,10 +1516,13 @@
     <t xml:space="preserve">Hints, level 3 (all three strategies)</t>
   </si>
   <si>
-    <t xml:space="preserve">Not an overgeneralisation but a validity risk: the hint gives the answer, so 'right after 3 hints' shows little.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keep as a model answer and treat as 'shown the answer' in the parent report, or remove level 3.</t>
+    <t xml:space="preserve">Worked example (this shows the answer): … = {word}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADDRESSED (pending your review): level 3 is now a labelled worked example. The app records that the answer was shown, reports it to the parent as such, never counts what follows as independent, and makes the next word a new one tried without a hint first.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check the new wording on the Hints sheet.</t>
   </si>
   <si>
     <t xml:space="preserve">OG-7</t>
@@ -1348,13 +1531,13 @@
     <t xml:space="preserve">Journey design: practice words and the check after teaching</t>
   </si>
   <si>
-    <t xml:space="preserve">All 12 practice words double; the 2 questions after teaching always double.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A child who learns 'always double' passes the check after teaching. Over-doubling would only show at the next diagnostic question.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add at least one 'must not double' word to practice and to the check after teaching (content change, needs approval).</t>
+    <t xml:space="preserve">All 12 practice words double. The check after teaching now includes a 'must not double' word (new contrasts spl.infl.26–31).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PARTLY ADDRESSED (pending your review): a child who learns 'always double' no longer passes the check after teaching. Practice itself still contains only doubling words.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decide whether practice also needs 'must not double' words (content change, needs approval).</t>
   </si>
   <si>
     <t xml:space="preserve">OG-8</t>
@@ -2036,23 +2219,23 @@
         <v>30</v>
       </c>
       <c r="B2" s="10" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C2" s="10" t="n">
-        <f aca="false">COUNTA(Questions!$N$2:$N$11)</f>
+        <f aca="false">COUNTA(Questions!$N$2:$N$17)</f>
         <v>0</v>
       </c>
       <c r="D2" s="10" t="n">
-        <f aca="false">COUNTIF(Questions!$N$2:$N$11,"Approve")+COUNTIF(Questions!$N$2:$N$11,"Approve with changes")</f>
+        <f aca="false">COUNTIF(Questions!$N$2:$N$17,"Approve")+COUNTIF(Questions!$N$2:$N$17,"Approve with changes")</f>
         <v>0</v>
       </c>
       <c r="E2" s="10" t="n">
-        <f aca="false">COUNTIF(Questions!$N$2:$N$11,"Reject")</f>
+        <f aca="false">COUNTIF(Questions!$N$2:$N$17,"Reject")</f>
         <v>0</v>
       </c>
       <c r="F2" s="10" t="n">
         <f aca="false">B2-C2</f>
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2156,23 +2339,23 @@
         <v>35</v>
       </c>
       <c r="B7" s="10" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="C7" s="10" t="n">
-        <f aca="false">COUNTA('Parent wording'!$F$2:$F$41)</f>
+        <f aca="false">COUNTA('Parent wording'!$F$2:$F$53)</f>
         <v>0</v>
       </c>
       <c r="D7" s="10" t="n">
-        <f aca="false">COUNTIF('Parent wording'!$F$2:$F$41,"Approve")+COUNTIF('Parent wording'!$F$2:$F$41,"Approve with changes")</f>
+        <f aca="false">COUNTIF('Parent wording'!$F$2:$F$53,"Approve")+COUNTIF('Parent wording'!$F$2:$F$53,"Approve with changes")</f>
         <v>0</v>
       </c>
       <c r="E7" s="10" t="n">
-        <f aca="false">COUNTIF('Parent wording'!$F$2:$F$41,"Reject")</f>
+        <f aca="false">COUNTIF('Parent wording'!$F$2:$F$53,"Reject")</f>
         <v>0</v>
       </c>
       <c r="F7" s="10" t="n">
         <f aca="false">B7-C7</f>
-        <v>40</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2205,7 +2388,7 @@
       </c>
       <c r="B9" s="11" t="n">
         <f aca="false">SUM(B2:B8)</f>
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="C9" s="11" t="n">
         <f aca="false">SUM(C2:C8)</f>
@@ -2221,7 +2404,7 @@
       </c>
       <c r="F9" s="11" t="n">
         <f aca="false">SUM(F2:F8)</f>
-        <v>97</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2229,7 +2412,7 @@
         <v>38</v>
       </c>
       <c r="D11" s="12" t="n">
-        <f aca="false">COUNTIF(Questions!$N$2:$N$11,"Approve")+COUNTIF(Questions!$N$2:$N$11,"Approve with changes")</f>
+        <f aca="false">COUNTIF(Questions!$N$2:$N$17,"Approve")+COUNTIF(Questions!$N$2:$N$17,"Approve with changes")</f>
         <v>0</v>
       </c>
     </row>
@@ -2264,7 +2447,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -2768,9 +2951,267 @@
       <c r="P11" s="16"/>
       <c r="Q11" s="16"/>
     </row>
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="F12" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="G12" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="H12" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="J12" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="K12" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="L12" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="M12" s="16"/>
+      <c r="N12" s="16"/>
+      <c r="O12" s="16"/>
+      <c r="P12" s="16"/>
+      <c r="Q12" s="16"/>
+    </row>
+    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="F13" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="G13" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="H13" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="J13" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="K13" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="L13" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="M13" s="16"/>
+      <c r="N13" s="16"/>
+      <c r="O13" s="16"/>
+      <c r="P13" s="16"/>
+      <c r="Q13" s="16"/>
+    </row>
+    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="F14" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="G14" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="H14" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="J14" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="K14" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="L14" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="M14" s="16"/>
+      <c r="N14" s="16"/>
+      <c r="O14" s="16"/>
+      <c r="P14" s="16"/>
+      <c r="Q14" s="16"/>
+    </row>
+    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="E15" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="F15" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="G15" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="H15" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="I15" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="J15" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="K15" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="L15" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="M15" s="16"/>
+      <c r="N15" s="16"/>
+      <c r="O15" s="16"/>
+      <c r="P15" s="16"/>
+      <c r="Q15" s="16"/>
+    </row>
+    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>148</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="F16" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="G16" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="H16" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="I16" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="J16" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="K16" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="L16" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="M16" s="16"/>
+      <c r="N16" s="16"/>
+      <c r="O16" s="16"/>
+      <c r="P16" s="16"/>
+      <c r="Q16" s="16"/>
+    </row>
+    <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="F17" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="G17" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="H17" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="J17" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="K17" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="L17" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="M17" s="16"/>
+      <c r="N17" s="16"/>
+      <c r="O17" s="16"/>
+      <c r="P17" s="16"/>
+      <c r="Q17" s="16"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N2:N11" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N2:N17" type="list">
       <formula1>"Approve,Approve with changes,Reject,Needs discussion"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2810,34 +3251,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>125</v>
+        <v>157</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>126</v>
+        <v>158</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>127</v>
+        <v>159</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>128</v>
+        <v>160</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>129</v>
+        <v>161</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>130</v>
+        <v>162</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>131</v>
+        <v>163</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>132</v>
+        <v>164</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>133</v>
+        <v>165</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>134</v>
+        <v>166</v>
       </c>
       <c r="K1" s="9" t="s">
         <v>54</v>
@@ -2854,106 +3295,106 @@
     </row>
     <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>135</v>
+        <v>167</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>136</v>
+        <v>168</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>137</v>
+        <v>169</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>138</v>
+        <v>170</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>139</v>
+        <v>171</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>140</v>
+        <v>172</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>141</v>
+        <v>173</v>
       </c>
       <c r="H2" s="14" t="s">
-        <v>142</v>
+        <v>174</v>
       </c>
       <c r="I2" s="15" t="s">
-        <v>143</v>
+        <v>175</v>
       </c>
       <c r="J2" s="14" t="s">
-        <v>144</v>
+        <v>176</v>
       </c>
       <c r="K2" s="16"/>
       <c r="L2" s="16"/>
       <c r="M2" s="16"/>
       <c r="N2" s="16"/>
     </row>
-    <row r="3" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>145</v>
+        <v>177</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>146</v>
+        <v>178</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>147</v>
+        <v>179</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>148</v>
+        <v>180</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>149</v>
+        <v>181</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>150</v>
+        <v>182</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>151</v>
+        <v>183</v>
       </c>
       <c r="H3" s="14" t="s">
-        <v>152</v>
+        <v>184</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>153</v>
+        <v>185</v>
       </c>
       <c r="J3" s="14" t="s">
-        <v>144</v>
+        <v>176</v>
       </c>
       <c r="K3" s="16"/>
       <c r="L3" s="16"/>
       <c r="M3" s="16"/>
       <c r="N3" s="16"/>
     </row>
-    <row r="4" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>154</v>
+        <v>186</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>155</v>
+        <v>187</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>156</v>
+        <v>188</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>157</v>
+        <v>189</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>158</v>
+        <v>190</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>159</v>
+        <v>191</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>160</v>
+        <v>192</v>
       </c>
       <c r="H4" s="14" t="s">
-        <v>161</v>
+        <v>193</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>162</v>
+        <v>194</v>
       </c>
       <c r="J4" s="14" t="s">
-        <v>144</v>
+        <v>176</v>
       </c>
       <c r="K4" s="16"/>
       <c r="L4" s="16"/>
@@ -2997,22 +3438,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>163</v>
+        <v>195</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>164</v>
+        <v>196</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>165</v>
+        <v>197</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>166</v>
+        <v>198</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>167</v>
+        <v>199</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>168</v>
+        <v>200</v>
       </c>
       <c r="G1" s="9" t="s">
         <v>54</v>
@@ -3029,19 +3470,19 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>135</v>
+        <v>167</v>
       </c>
       <c r="B2" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>169</v>
+        <v>201</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>169</v>
+        <v>201</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>169</v>
+        <v>201</v>
       </c>
       <c r="F2" s="14"/>
       <c r="G2" s="16"/>
@@ -3051,19 +3492,19 @@
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>135</v>
+        <v>167</v>
       </c>
       <c r="B3" s="14" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>170</v>
+        <v>202</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>171</v>
+        <v>203</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>172</v>
+        <v>204</v>
       </c>
       <c r="F3" s="14"/>
       <c r="G3" s="16"/>
@@ -3071,24 +3512,24 @@
       <c r="I3" s="16"/>
       <c r="J3" s="16"/>
     </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>135</v>
+        <v>167</v>
       </c>
       <c r="B4" s="14" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>173</v>
+        <v>205</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>174</v>
+        <v>206</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>175</v>
+        <v>207</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>176</v>
+        <v>208</v>
       </c>
       <c r="G4" s="16"/>
       <c r="H4" s="16"/>
@@ -3097,22 +3538,22 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>145</v>
+        <v>177</v>
       </c>
       <c r="B5" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>177</v>
+        <v>209</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>178</v>
+        <v>210</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>179</v>
+        <v>211</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>180</v>
+        <v>212</v>
       </c>
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
@@ -3121,46 +3562,46 @@
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>145</v>
+        <v>177</v>
       </c>
       <c r="B6" s="14" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>181</v>
+        <v>213</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>182</v>
+        <v>214</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>182</v>
+        <v>214</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>183</v>
+        <v>215</v>
       </c>
       <c r="G6" s="16"/>
       <c r="H6" s="16"/>
       <c r="I6" s="16"/>
       <c r="J6" s="16"/>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>145</v>
+        <v>177</v>
       </c>
       <c r="B7" s="14" t="n">
         <v>3</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>184</v>
+        <v>216</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>185</v>
+        <v>217</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>186</v>
+        <v>218</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>187</v>
+        <v>219</v>
       </c>
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
@@ -3169,19 +3610,19 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>154</v>
+        <v>186</v>
       </c>
       <c r="B8" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>188</v>
+        <v>220</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>189</v>
+        <v>221</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>190</v>
+        <v>222</v>
       </c>
       <c r="F8" s="14"/>
       <c r="G8" s="16"/>
@@ -3191,19 +3632,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>154</v>
+        <v>186</v>
       </c>
       <c r="B9" s="14" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>191</v>
+        <v>223</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>192</v>
+        <v>224</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>192</v>
+        <v>224</v>
       </c>
       <c r="F9" s="14"/>
       <c r="G9" s="16"/>
@@ -3211,24 +3652,24 @@
       <c r="I9" s="16"/>
       <c r="J9" s="16"/>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>154</v>
+        <v>186</v>
       </c>
       <c r="B10" s="14" t="n">
         <v>3</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>184</v>
+        <v>225</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>185</v>
+        <v>226</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>186</v>
+        <v>227</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>187</v>
+        <v>208</v>
       </c>
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
@@ -3282,25 +3723,25 @@
         <v>42</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>193</v>
+        <v>228</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>194</v>
+        <v>229</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>195</v>
+        <v>230</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>196</v>
+        <v>231</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>197</v>
+        <v>232</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>198</v>
+        <v>233</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>168</v>
+        <v>200</v>
       </c>
       <c r="J1" s="9" t="s">
         <v>54</v>
@@ -3320,25 +3761,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>199</v>
+        <v>234</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>200</v>
+        <v>235</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>201</v>
+        <v>236</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>202</v>
+        <v>237</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>203</v>
+        <v>238</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>204</v>
+        <v>239</v>
       </c>
       <c r="H2" s="14" t="s">
-        <v>205</v>
+        <v>240</v>
       </c>
       <c r="I2" s="14"/>
       <c r="J2" s="16"/>
@@ -3351,25 +3792,25 @@
         <v>2</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>206</v>
+        <v>241</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>207</v>
+        <v>242</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>201</v>
+        <v>236</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>208</v>
+        <v>243</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>209</v>
+        <v>244</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>210</v>
+        <v>245</v>
       </c>
       <c r="H3" s="14" t="s">
-        <v>211</v>
+        <v>246</v>
       </c>
       <c r="I3" s="14"/>
       <c r="J3" s="16"/>
@@ -3382,25 +3823,25 @@
         <v>3</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>212</v>
+        <v>247</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>213</v>
+        <v>248</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>214</v>
+        <v>249</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>215</v>
+        <v>250</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>216</v>
+        <v>251</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>217</v>
+        <v>252</v>
       </c>
       <c r="H4" s="14" t="s">
-        <v>218</v>
+        <v>253</v>
       </c>
       <c r="I4" s="14"/>
       <c r="J4" s="16"/>
@@ -3413,25 +3854,25 @@
         <v>4</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>219</v>
+        <v>254</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>220</v>
+        <v>255</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>201</v>
+        <v>236</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>221</v>
+        <v>256</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>222</v>
+        <v>257</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>223</v>
+        <v>258</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>224</v>
+        <v>259</v>
       </c>
       <c r="I5" s="14"/>
       <c r="J5" s="16"/>
@@ -3444,25 +3885,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>225</v>
+        <v>260</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>226</v>
+        <v>261</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>201</v>
+        <v>236</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>227</v>
+        <v>262</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>228</v>
+        <v>263</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>229</v>
+        <v>264</v>
       </c>
       <c r="H6" s="14" t="s">
-        <v>230</v>
+        <v>265</v>
       </c>
       <c r="I6" s="14"/>
       <c r="J6" s="16"/>
@@ -3475,25 +3916,25 @@
         <v>6</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>231</v>
+        <v>266</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>232</v>
+        <v>267</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>201</v>
+        <v>236</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>233</v>
+        <v>268</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>234</v>
+        <v>269</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>235</v>
+        <v>270</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>236</v>
+        <v>271</v>
       </c>
       <c r="I7" s="14"/>
       <c r="J7" s="16"/>
@@ -3506,25 +3947,25 @@
         <v>7</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>237</v>
+        <v>272</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>238</v>
+        <v>273</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>201</v>
+        <v>236</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>239</v>
+        <v>274</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>240</v>
+        <v>275</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>241</v>
+        <v>276</v>
       </c>
       <c r="H8" s="14" t="s">
-        <v>242</v>
+        <v>277</v>
       </c>
       <c r="I8" s="14"/>
       <c r="J8" s="16"/>
@@ -3537,26 +3978,26 @@
         <v>8</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>243</v>
+        <v>278</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>244</v>
+        <v>279</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>201</v>
+        <v>236</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>245</v>
+        <v>280</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>246</v>
+        <v>281</v>
       </c>
       <c r="G9" s="14"/>
       <c r="H9" s="14" t="s">
-        <v>247</v>
+        <v>282</v>
       </c>
       <c r="I9" s="15" t="s">
-        <v>248</v>
+        <v>283</v>
       </c>
       <c r="J9" s="16"/>
       <c r="K9" s="16"/>
@@ -3568,25 +4009,25 @@
         <v>9</v>
       </c>
       <c r="B10" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="D10" s="14" t="s">
         <v>249</v>
       </c>
-      <c r="C10" s="14" t="s">
-        <v>250</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>214</v>
-      </c>
       <c r="E10" s="14" t="s">
-        <v>251</v>
+        <v>286</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>252</v>
+        <v>287</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>253</v>
+        <v>288</v>
       </c>
       <c r="H10" s="14" t="s">
-        <v>254</v>
+        <v>289</v>
       </c>
       <c r="I10" s="14"/>
       <c r="J10" s="16"/>
@@ -3599,25 +4040,25 @@
         <v>10</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>255</v>
+        <v>290</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>256</v>
+        <v>291</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>201</v>
+        <v>236</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>257</v>
+        <v>292</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>258</v>
+        <v>293</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>259</v>
+        <v>294</v>
       </c>
       <c r="H11" s="14" t="s">
-        <v>260</v>
+        <v>295</v>
       </c>
       <c r="I11" s="14"/>
       <c r="J11" s="16"/>
@@ -3630,26 +4071,26 @@
         <v>11</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>261</v>
+        <v>296</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>262</v>
+        <v>297</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>201</v>
+        <v>236</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>263</v>
+        <v>298</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>264</v>
+        <v>299</v>
       </c>
       <c r="G12" s="14"/>
       <c r="H12" s="14" t="s">
-        <v>265</v>
+        <v>300</v>
       </c>
       <c r="I12" s="15" t="s">
-        <v>266</v>
+        <v>301</v>
       </c>
       <c r="J12" s="16"/>
       <c r="K12" s="16"/>
@@ -3661,25 +4102,25 @@
         <v>12</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>267</v>
+        <v>302</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>268</v>
+        <v>303</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>201</v>
+        <v>236</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>269</v>
+        <v>304</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>270</v>
+        <v>305</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>271</v>
+        <v>306</v>
       </c>
       <c r="H13" s="14" t="s">
-        <v>272</v>
+        <v>307</v>
       </c>
       <c r="I13" s="14"/>
       <c r="J13" s="16"/>
@@ -3689,12 +4130,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="5" t="s">
-        <v>273</v>
+        <v>308</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="17" t="s">
-        <v>274</v>
+        <v>309</v>
       </c>
       <c r="C16" s="17"/>
       <c r="D16" s="17"/>
@@ -3743,19 +4184,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>275</v>
+        <v>310</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>276</v>
+        <v>311</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>277</v>
+        <v>312</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>278</v>
+        <v>313</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>279</v>
+        <v>314</v>
       </c>
       <c r="F1" s="9" t="s">
         <v>54</v>
@@ -3772,16 +4213,16 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>280</v>
+        <v>315</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>281</v>
+        <v>316</v>
       </c>
       <c r="C2" s="14" t="n">
         <v>5</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>282</v>
+        <v>317</v>
       </c>
       <c r="E2" s="16"/>
       <c r="F2" s="16"/>
@@ -3791,16 +4232,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>280</v>
+        <v>315</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>283</v>
+        <v>318</v>
       </c>
       <c r="C3" s="14" t="n">
         <v>4</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>284</v>
+        <v>319</v>
       </c>
       <c r="E3" s="16"/>
       <c r="F3" s="16"/>
@@ -3810,16 +4251,16 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>280</v>
+        <v>315</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>285</v>
+        <v>320</v>
       </c>
       <c r="C4" s="14" t="n">
         <v>3</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>286</v>
+        <v>321</v>
       </c>
       <c r="E4" s="16"/>
       <c r="F4" s="16"/>
@@ -3829,16 +4270,16 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>280</v>
+        <v>315</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>287</v>
+        <v>322</v>
       </c>
       <c r="C5" s="14" t="n">
         <v>2</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>288</v>
+        <v>323</v>
       </c>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
@@ -3848,16 +4289,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>280</v>
+        <v>315</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>289</v>
+        <v>324</v>
       </c>
       <c r="C6" s="14" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>290</v>
+        <v>325</v>
       </c>
       <c r="E6" s="16"/>
       <c r="F6" s="16"/>
@@ -3867,16 +4308,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>280</v>
+        <v>315</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>291</v>
+        <v>326</v>
       </c>
       <c r="C7" s="14" t="n">
         <v>3</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>292</v>
+        <v>327</v>
       </c>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
@@ -3886,16 +4327,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>280</v>
+        <v>315</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>293</v>
+        <v>328</v>
       </c>
       <c r="C8" s="14" t="n">
         <v>7</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>294</v>
+        <v>329</v>
       </c>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
@@ -3905,16 +4346,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>280</v>
+        <v>315</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>295</v>
+        <v>330</v>
       </c>
       <c r="C9" s="14" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>296</v>
+        <v>331</v>
       </c>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
@@ -3924,16 +4365,16 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>297</v>
+        <v>332</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>298</v>
+        <v>333</v>
       </c>
       <c r="C10" s="14" t="n">
         <v>4</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>299</v>
+        <v>334</v>
       </c>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
@@ -3943,16 +4384,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>297</v>
+        <v>332</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>300</v>
+        <v>335</v>
       </c>
       <c r="C11" s="14" t="n">
         <v>1</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>301</v>
+        <v>336</v>
       </c>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
@@ -3962,16 +4403,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>297</v>
+        <v>332</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>302</v>
+        <v>337</v>
       </c>
       <c r="C12" s="14" t="n">
         <v>8</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>303</v>
+        <v>338</v>
       </c>
       <c r="E12" s="16"/>
       <c r="F12" s="16"/>
@@ -3981,16 +4422,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>297</v>
+        <v>332</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>304</v>
+        <v>339</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>305</v>
+        <v>340</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>306</v>
+        <v>341</v>
       </c>
       <c r="E13" s="16"/>
       <c r="F13" s="16"/>
@@ -4000,16 +4441,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>297</v>
+        <v>332</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>307</v>
+        <v>342</v>
       </c>
       <c r="C14" s="14" t="n">
         <v>2</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>308</v>
+        <v>343</v>
       </c>
       <c r="E14" s="16"/>
       <c r="F14" s="16"/>
@@ -4019,16 +4460,16 @@
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>297</v>
+        <v>332</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>309</v>
+        <v>344</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>310</v>
+        <v>345</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>311</v>
+        <v>346</v>
       </c>
       <c r="E15" s="16"/>
       <c r="F15" s="16"/>
@@ -4038,16 +4479,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>312</v>
+        <v>347</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>313</v>
+        <v>348</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>314</v>
+        <v>349</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>315</v>
+        <v>350</v>
       </c>
       <c r="E16" s="16"/>
       <c r="F16" s="16"/>
@@ -4057,7 +4498,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>316</v>
+        <v>351</v>
       </c>
     </row>
   </sheetData>
@@ -4082,7 +4523,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -4098,19 +4539,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>317</v>
+        <v>352</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>318</v>
+        <v>353</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>319</v>
+        <v>354</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>320</v>
+        <v>355</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>168</v>
+        <v>200</v>
       </c>
       <c r="F1" s="9" t="s">
         <v>54</v>
@@ -4127,16 +4568,16 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>321</v>
+        <v>356</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>322</v>
+        <v>357</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>323</v>
+        <v>358</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>324</v>
+        <v>359</v>
       </c>
       <c r="E2" s="14"/>
       <c r="F2" s="16"/>
@@ -4146,16 +4587,16 @@
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>321</v>
+        <v>356</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>322</v>
+        <v>357</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>325</v>
+        <v>360</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>324</v>
+        <v>359</v>
       </c>
       <c r="E3" s="14"/>
       <c r="F3" s="16"/>
@@ -4165,16 +4606,16 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>321</v>
+        <v>356</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>326</v>
+        <v>361</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>327</v>
+        <v>362</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>328</v>
+        <v>363</v>
       </c>
       <c r="E4" s="14"/>
       <c r="F4" s="16"/>
@@ -4184,16 +4625,16 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>321</v>
+        <v>356</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>326</v>
+        <v>361</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>329</v>
+        <v>364</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>328</v>
+        <v>363</v>
       </c>
       <c r="E5" s="14"/>
       <c r="F5" s="16"/>
@@ -4203,19 +4644,19 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>321</v>
+        <v>356</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>326</v>
+        <v>361</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>330</v>
+        <v>365</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>328</v>
+        <v>363</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>331</v>
+        <v>366</v>
       </c>
       <c r="F6" s="16"/>
       <c r="G6" s="16"/>
@@ -4224,16 +4665,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>321</v>
+        <v>356</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>332</v>
+        <v>367</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>333</v>
+        <v>368</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>328</v>
+        <v>363</v>
       </c>
       <c r="E7" s="14"/>
       <c r="F7" s="16"/>
@@ -4243,19 +4684,19 @@
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>321</v>
+        <v>356</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>334</v>
+        <v>369</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>335</v>
+        <v>370</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>336</v>
+        <v>371</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>337</v>
+        <v>372</v>
       </c>
       <c r="F8" s="16"/>
       <c r="G8" s="16"/>
@@ -4264,16 +4705,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>321</v>
+        <v>356</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>334</v>
+        <v>369</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>338</v>
+        <v>373</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>336</v>
+        <v>371</v>
       </c>
       <c r="E9" s="14"/>
       <c r="F9" s="16"/>
@@ -4283,16 +4724,16 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>321</v>
+        <v>356</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>334</v>
+        <v>369</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>339</v>
+        <v>374</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>336</v>
+        <v>371</v>
       </c>
       <c r="E10" s="14"/>
       <c r="F10" s="16"/>
@@ -4302,16 +4743,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>321</v>
+        <v>356</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>340</v>
+        <v>375</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>341</v>
+        <v>376</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>328</v>
+        <v>363</v>
       </c>
       <c r="E11" s="14"/>
       <c r="F11" s="16"/>
@@ -4321,16 +4762,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>321</v>
+        <v>356</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>342</v>
+        <v>377</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>343</v>
+        <v>378</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>328</v>
+        <v>363</v>
       </c>
       <c r="E12" s="14"/>
       <c r="F12" s="16"/>
@@ -4338,59 +4779,63 @@
       <c r="H12" s="16"/>
       <c r="I12" s="16"/>
     </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>321</v>
+        <v>356</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>344</v>
+        <v>377</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>345</v>
+        <v>379</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>328</v>
-      </c>
-      <c r="E13" s="14"/>
+        <v>363</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>380</v>
+      </c>
       <c r="F13" s="16"/>
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
       <c r="I13" s="16"/>
     </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>321</v>
+        <v>356</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>344</v>
+        <v>381</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>346</v>
+        <v>382</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>328</v>
-      </c>
-      <c r="E14" s="14"/>
+        <v>363</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>383</v>
+      </c>
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
       <c r="I14" s="16"/>
     </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>321</v>
+        <v>356</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>344</v>
+        <v>384</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>347</v>
+        <v>385</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>328</v>
+        <v>363</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>348</v>
+        <v>386</v>
       </c>
       <c r="F15" s="16"/>
       <c r="G15" s="16"/>
@@ -4399,18 +4844,20 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>321</v>
+        <v>356</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>344</v>
+        <v>377</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>349</v>
+        <v>387</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>328</v>
-      </c>
-      <c r="E16" s="14"/>
+        <v>363</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>386</v>
+      </c>
       <c r="F16" s="16"/>
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
@@ -4418,56 +4865,58 @@
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>351</v>
+        <v>375</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>352</v>
+        <v>388</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>353</v>
+        <v>363</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>354</v>
+        <v>389</v>
       </c>
       <c r="F17" s="16"/>
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
       <c r="I17" s="16"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>355</v>
+        <v>369</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>356</v>
+        <v>390</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>353</v>
-      </c>
-      <c r="E18" s="14"/>
+        <v>371</v>
+      </c>
+      <c r="E18" s="15" t="s">
+        <v>391</v>
+      </c>
       <c r="F18" s="16"/>
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
       <c r="I18" s="16"/>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>355</v>
+        <v>392</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>357</v>
+        <v>393</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>353</v>
+        <v>363</v>
       </c>
       <c r="E19" s="14"/>
       <c r="F19" s="16"/>
@@ -4475,18 +4924,18 @@
       <c r="H19" s="16"/>
       <c r="I19" s="16"/>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>355</v>
+        <v>392</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>358</v>
+        <v>394</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>353</v>
+        <v>363</v>
       </c>
       <c r="E20" s="14"/>
       <c r="F20" s="16"/>
@@ -4494,20 +4943,22 @@
       <c r="H20" s="16"/>
       <c r="I20" s="16"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>355</v>
+        <v>392</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>359</v>
+        <v>395</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>353</v>
-      </c>
-      <c r="E21" s="14"/>
+        <v>363</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>396</v>
+      </c>
       <c r="F21" s="16"/>
       <c r="G21" s="16"/>
       <c r="H21" s="16"/>
@@ -4515,16 +4966,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>355</v>
+        <v>392</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>360</v>
+        <v>397</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>353</v>
+        <v>363</v>
       </c>
       <c r="E22" s="14"/>
       <c r="F22" s="16"/>
@@ -4534,19 +4985,19 @@
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="s">
-        <v>350</v>
+        <v>398</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>355</v>
+        <v>399</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>361</v>
+        <v>400</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>353</v>
+        <v>401</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>362</v>
+        <v>402</v>
       </c>
       <c r="F23" s="16"/>
       <c r="G23" s="16"/>
@@ -4555,16 +5006,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="14" t="s">
-        <v>350</v>
+        <v>398</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>355</v>
+        <v>403</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>363</v>
+        <v>404</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>353</v>
+        <v>401</v>
       </c>
       <c r="E24" s="14"/>
       <c r="F24" s="16"/>
@@ -4574,16 +5025,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>350</v>
+        <v>398</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>355</v>
+        <v>403</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>364</v>
+        <v>405</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>353</v>
+        <v>401</v>
       </c>
       <c r="E25" s="14"/>
       <c r="F25" s="16"/>
@@ -4591,18 +5042,18 @@
       <c r="H25" s="16"/>
       <c r="I25" s="16"/>
     </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="s">
-        <v>350</v>
+        <v>398</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>355</v>
+        <v>403</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>365</v>
+        <v>406</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>353</v>
+        <v>401</v>
       </c>
       <c r="E26" s="14"/>
       <c r="F26" s="16"/>
@@ -4612,16 +5063,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="s">
-        <v>350</v>
+        <v>398</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>355</v>
+        <v>403</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>366</v>
+        <v>407</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>353</v>
+        <v>401</v>
       </c>
       <c r="E27" s="14"/>
       <c r="F27" s="16"/>
@@ -4631,16 +5082,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
-        <v>350</v>
+        <v>398</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>367</v>
+        <v>403</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>368</v>
+        <v>408</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>353</v>
+        <v>401</v>
       </c>
       <c r="E28" s="14"/>
       <c r="F28" s="16"/>
@@ -4650,19 +5101,19 @@
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="s">
-        <v>350</v>
+        <v>398</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>369</v>
+        <v>403</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>370</v>
+        <v>409</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>353</v>
+        <v>401</v>
       </c>
       <c r="E29" s="15" t="s">
-        <v>371</v>
+        <v>410</v>
       </c>
       <c r="F29" s="16"/>
       <c r="G29" s="16"/>
@@ -4671,16 +5122,16 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="14" t="s">
-        <v>350</v>
+        <v>398</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>372</v>
+        <v>403</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>373</v>
+        <v>411</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>353</v>
+        <v>401</v>
       </c>
       <c r="E30" s="14"/>
       <c r="F30" s="16"/>
@@ -4688,18 +5139,18 @@
       <c r="H30" s="16"/>
       <c r="I30" s="16"/>
     </row>
-    <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="14" t="s">
-        <v>350</v>
+        <v>398</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>374</v>
+        <v>403</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>375</v>
+        <v>412</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>353</v>
+        <v>401</v>
       </c>
       <c r="E31" s="14"/>
       <c r="F31" s="16"/>
@@ -4707,18 +5158,18 @@
       <c r="H31" s="16"/>
       <c r="I31" s="16"/>
     </row>
-    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="14" t="s">
-        <v>350</v>
+        <v>398</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>376</v>
+        <v>403</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>377</v>
+        <v>413</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>353</v>
+        <v>401</v>
       </c>
       <c r="E32" s="14"/>
       <c r="F32" s="16"/>
@@ -4726,18 +5177,18 @@
       <c r="H32" s="16"/>
       <c r="I32" s="16"/>
     </row>
-    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>350</v>
+        <v>398</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>378</v>
+        <v>414</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>379</v>
+        <v>415</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
       <c r="E33" s="14"/>
       <c r="F33" s="16"/>
@@ -4745,20 +5196,22 @@
       <c r="H33" s="16"/>
       <c r="I33" s="16"/>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
-        <v>350</v>
+        <v>398</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>378</v>
+        <v>416</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>380</v>
+        <v>417</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>328</v>
-      </c>
-      <c r="E34" s="14"/>
+        <v>401</v>
+      </c>
+      <c r="E34" s="15" t="s">
+        <v>418</v>
+      </c>
       <c r="F34" s="16"/>
       <c r="G34" s="16"/>
       <c r="H34" s="16"/>
@@ -4766,16 +5219,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="14" t="s">
-        <v>350</v>
+        <v>398</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>381</v>
+        <v>419</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>382</v>
+        <v>420</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
       <c r="E35" s="14"/>
       <c r="F35" s="16"/>
@@ -4785,16 +5238,16 @@
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="14" t="s">
-        <v>350</v>
+        <v>398</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>383</v>
+        <v>421</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>384</v>
+        <v>422</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
       <c r="E36" s="14"/>
       <c r="F36" s="16"/>
@@ -4802,18 +5255,18 @@
       <c r="H36" s="16"/>
       <c r="I36" s="16"/>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="14" t="s">
-        <v>350</v>
+        <v>398</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>383</v>
+        <v>423</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>385</v>
+        <v>424</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
       <c r="E37" s="14"/>
       <c r="F37" s="16"/>
@@ -4821,18 +5274,18 @@
       <c r="H37" s="16"/>
       <c r="I37" s="16"/>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="14" t="s">
-        <v>350</v>
+        <v>398</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>383</v>
+        <v>425</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>386</v>
+        <v>426</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>328</v>
+        <v>363</v>
       </c>
       <c r="E38" s="14"/>
       <c r="F38" s="16"/>
@@ -4842,64 +5295,308 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="14" t="s">
-        <v>350</v>
+        <v>398</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>383</v>
+        <v>425</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>387</v>
+        <v>427</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>328</v>
-      </c>
-      <c r="E39" s="14"/>
+        <v>363</v>
+      </c>
+      <c r="E39" s="15" t="s">
+        <v>428</v>
+      </c>
       <c r="F39" s="16"/>
       <c r="G39" s="16"/>
       <c r="H39" s="16"/>
       <c r="I39" s="16"/>
     </row>
-    <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="14" t="s">
-        <v>350</v>
+        <v>398</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>388</v>
+        <v>421</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>389</v>
+        <v>429</v>
       </c>
       <c r="D40" s="14" t="s">
-        <v>353</v>
-      </c>
-      <c r="E40" s="14"/>
+        <v>401</v>
+      </c>
+      <c r="E40" s="15" t="s">
+        <v>430</v>
+      </c>
       <c r="F40" s="16"/>
       <c r="G40" s="16"/>
       <c r="H40" s="16"/>
       <c r="I40" s="16"/>
     </row>
-    <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="14" t="s">
-        <v>350</v>
+        <v>398</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>390</v>
+        <v>421</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>391</v>
+        <v>431</v>
       </c>
       <c r="D41" s="14" t="s">
-        <v>353</v>
-      </c>
-      <c r="E41" s="14"/>
+        <v>401</v>
+      </c>
+      <c r="E41" s="15" t="s">
+        <v>386</v>
+      </c>
       <c r="F41" s="16"/>
       <c r="G41" s="16"/>
       <c r="H41" s="16"/>
       <c r="I41" s="16"/>
     </row>
+    <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="14" t="s">
+        <v>398</v>
+      </c>
+      <c r="B42" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="C42" s="14" t="s">
+        <v>432</v>
+      </c>
+      <c r="D42" s="14" t="s">
+        <v>401</v>
+      </c>
+      <c r="E42" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="F42" s="16"/>
+      <c r="G42" s="16"/>
+      <c r="H42" s="16"/>
+      <c r="I42" s="16"/>
+    </row>
+    <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="14" t="s">
+        <v>398</v>
+      </c>
+      <c r="B43" s="14" t="s">
+        <v>403</v>
+      </c>
+      <c r="C43" s="14" t="s">
+        <v>434</v>
+      </c>
+      <c r="D43" s="14" t="s">
+        <v>401</v>
+      </c>
+      <c r="E43" s="15" t="s">
+        <v>435</v>
+      </c>
+      <c r="F43" s="16"/>
+      <c r="G43" s="16"/>
+      <c r="H43" s="16"/>
+      <c r="I43" s="16"/>
+    </row>
+    <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="14" t="s">
+        <v>398</v>
+      </c>
+      <c r="B44" s="14" t="s">
+        <v>436</v>
+      </c>
+      <c r="C44" s="14" t="s">
+        <v>437</v>
+      </c>
+      <c r="D44" s="14" t="s">
+        <v>401</v>
+      </c>
+      <c r="E44" s="15" t="s">
+        <v>386</v>
+      </c>
+      <c r="F44" s="16"/>
+      <c r="G44" s="16"/>
+      <c r="H44" s="16"/>
+      <c r="I44" s="16"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="14" t="s">
+        <v>398</v>
+      </c>
+      <c r="B45" s="14" t="s">
+        <v>425</v>
+      </c>
+      <c r="C45" s="14" t="s">
+        <v>438</v>
+      </c>
+      <c r="D45" s="14" t="s">
+        <v>363</v>
+      </c>
+      <c r="E45" s="14"/>
+      <c r="F45" s="16"/>
+      <c r="G45" s="16"/>
+      <c r="H45" s="16"/>
+      <c r="I45" s="16"/>
+    </row>
+    <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="14" t="s">
+        <v>398</v>
+      </c>
+      <c r="B46" s="14" t="s">
+        <v>439</v>
+      </c>
+      <c r="C46" s="14" t="s">
+        <v>440</v>
+      </c>
+      <c r="D46" s="14" t="s">
+        <v>363</v>
+      </c>
+      <c r="E46" s="15" t="s">
+        <v>441</v>
+      </c>
+      <c r="F46" s="16"/>
+      <c r="G46" s="16"/>
+      <c r="H46" s="16"/>
+      <c r="I46" s="16"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="14" t="s">
+        <v>398</v>
+      </c>
+      <c r="B47" s="14" t="s">
+        <v>439</v>
+      </c>
+      <c r="C47" s="14" t="s">
+        <v>442</v>
+      </c>
+      <c r="D47" s="14" t="s">
+        <v>363</v>
+      </c>
+      <c r="E47" s="15" t="s">
+        <v>386</v>
+      </c>
+      <c r="F47" s="16"/>
+      <c r="G47" s="16"/>
+      <c r="H47" s="16"/>
+      <c r="I47" s="16"/>
+    </row>
+    <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="14" t="s">
+        <v>398</v>
+      </c>
+      <c r="B48" s="14" t="s">
+        <v>443</v>
+      </c>
+      <c r="C48" s="14" t="s">
+        <v>444</v>
+      </c>
+      <c r="D48" s="14" t="s">
+        <v>363</v>
+      </c>
+      <c r="E48" s="14"/>
+      <c r="F48" s="16"/>
+      <c r="G48" s="16"/>
+      <c r="H48" s="16"/>
+      <c r="I48" s="16"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="14" t="s">
+        <v>398</v>
+      </c>
+      <c r="B49" s="14" t="s">
+        <v>443</v>
+      </c>
+      <c r="C49" s="14" t="s">
+        <v>445</v>
+      </c>
+      <c r="D49" s="14" t="s">
+        <v>363</v>
+      </c>
+      <c r="E49" s="14"/>
+      <c r="F49" s="16"/>
+      <c r="G49" s="16"/>
+      <c r="H49" s="16"/>
+      <c r="I49" s="16"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="14" t="s">
+        <v>398</v>
+      </c>
+      <c r="B50" s="14" t="s">
+        <v>443</v>
+      </c>
+      <c r="C50" s="14" t="s">
+        <v>446</v>
+      </c>
+      <c r="D50" s="14" t="s">
+        <v>363</v>
+      </c>
+      <c r="E50" s="14"/>
+      <c r="F50" s="16"/>
+      <c r="G50" s="16"/>
+      <c r="H50" s="16"/>
+      <c r="I50" s="16"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="14" t="s">
+        <v>398</v>
+      </c>
+      <c r="B51" s="14" t="s">
+        <v>443</v>
+      </c>
+      <c r="C51" s="14" t="s">
+        <v>447</v>
+      </c>
+      <c r="D51" s="14" t="s">
+        <v>363</v>
+      </c>
+      <c r="E51" s="14"/>
+      <c r="F51" s="16"/>
+      <c r="G51" s="16"/>
+      <c r="H51" s="16"/>
+      <c r="I51" s="16"/>
+    </row>
+    <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="14" t="s">
+        <v>398</v>
+      </c>
+      <c r="B52" s="14" t="s">
+        <v>448</v>
+      </c>
+      <c r="C52" s="14" t="s">
+        <v>449</v>
+      </c>
+      <c r="D52" s="14" t="s">
+        <v>401</v>
+      </c>
+      <c r="E52" s="14"/>
+      <c r="F52" s="16"/>
+      <c r="G52" s="16"/>
+      <c r="H52" s="16"/>
+      <c r="I52" s="16"/>
+    </row>
+    <row r="53" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="14" t="s">
+        <v>398</v>
+      </c>
+      <c r="B53" s="14" t="s">
+        <v>450</v>
+      </c>
+      <c r="C53" s="14" t="s">
+        <v>451</v>
+      </c>
+      <c r="D53" s="14" t="s">
+        <v>401</v>
+      </c>
+      <c r="E53" s="14"/>
+      <c r="F53" s="16"/>
+      <c r="G53" s="16"/>
+      <c r="H53" s="16"/>
+      <c r="I53" s="16"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F41" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F53" type="list">
       <formula1>"Approve,Approve with changes,Reject,Needs discussion"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4935,19 +5632,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>392</v>
+        <v>452</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>393</v>
+        <v>453</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>394</v>
+        <v>454</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>395</v>
+        <v>455</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>396</v>
+        <v>456</v>
       </c>
       <c r="F1" s="9" t="s">
         <v>54</v>
@@ -4964,19 +5661,19 @@
     </row>
     <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>397</v>
+        <v>457</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>398</v>
+        <v>458</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>399</v>
+        <v>459</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>400</v>
+        <v>460</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>401</v>
+        <v>461</v>
       </c>
       <c r="F2" s="16"/>
       <c r="G2" s="16"/>
@@ -4985,19 +5682,19 @@
     </row>
     <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>402</v>
+        <v>462</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>403</v>
+        <v>463</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>404</v>
+        <v>464</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>405</v>
+        <v>465</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>406</v>
+        <v>466</v>
       </c>
       <c r="F3" s="16"/>
       <c r="G3" s="16"/>
@@ -5006,19 +5703,19 @@
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>407</v>
+        <v>467</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>408</v>
+        <v>468</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>409</v>
+        <v>469</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>410</v>
+        <v>470</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>411</v>
+        <v>471</v>
       </c>
       <c r="F4" s="16"/>
       <c r="G4" s="16"/>
@@ -5027,19 +5724,19 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>412</v>
+        <v>472</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>413</v>
+        <v>473</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>414</v>
+        <v>474</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>415</v>
+        <v>475</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>416</v>
+        <v>476</v>
       </c>
       <c r="F5" s="16"/>
       <c r="G5" s="16"/>
@@ -5048,40 +5745,40 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>417</v>
+        <v>477</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>418</v>
+        <v>478</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>419</v>
+        <v>479</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>420</v>
+        <v>480</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>421</v>
+        <v>481</v>
       </c>
       <c r="F6" s="16"/>
       <c r="G6" s="16"/>
       <c r="H6" s="16"/>
       <c r="I6" s="16"/>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>422</v>
+        <v>482</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>423</v>
+        <v>483</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>173</v>
+        <v>484</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>424</v>
+        <v>485</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>425</v>
+        <v>486</v>
       </c>
       <c r="F7" s="16"/>
       <c r="G7" s="16"/>
@@ -5090,19 +5787,19 @@
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>426</v>
+        <v>487</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>427</v>
+        <v>488</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>428</v>
+        <v>489</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>429</v>
+        <v>490</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>430</v>
+        <v>491</v>
       </c>
       <c r="F8" s="16"/>
       <c r="G8" s="16"/>
@@ -5111,19 +5808,19 @@
     </row>
     <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>431</v>
+        <v>492</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>432</v>
+        <v>493</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>433</v>
+        <v>494</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>434</v>
+        <v>495</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>435</v>
+        <v>496</v>
       </c>
       <c r="F9" s="16"/>
       <c r="G9" s="16"/>

</xml_diff>